<commit_message>
feat(ajout comment): Ajout des commentaire + notes
J'ai commencé a ajouter, il reste quelques trucs a modifier.
</commit_message>
<xml_diff>
--- a/Doc/X-Journal-de-Travail_ReynaudThomas.xlsx
+++ b/Doc/X-Journal-de-Travail_ReynaudThomas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk84vtk\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pk84vtk\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03866060-D5D4-4846-8A70-CDEFA96EA5F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C462DE8A-FE5D-436E-97FC-4D98F1362830}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2985" yWindow="2985" windowWidth="21600" windowHeight="11385" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="52">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -149,6 +149,54 @@
   </si>
   <si>
     <t>Reynaud Thomas</t>
+  </si>
+  <si>
+    <t>J'ai fais et terminé l'UI de la page d'accueil</t>
+  </si>
+  <si>
+    <t>J'ai rajouté des routes HTTP et montré aux profs.</t>
+  </si>
+  <si>
+    <t>J'ai commencé a faire les routes ainsi que des test pour faire la page détails</t>
+  </si>
+  <si>
+    <t>J'ai relié mon fichier .json test avec les 5 derniers ouvrages.</t>
+  </si>
+  <si>
+    <t>J'ai fais des changement dans les branches et je me suis mis sur ma propre branche afin de ne pas avoir d'influence sur la branche main. Mais il y avait des problèmes de conflit de versions</t>
+  </si>
+  <si>
+    <t>Le prof est venu nous voir afin de determiner notre avancement dans le projet et ils nous a corrigés sur quelques points mal executés</t>
+  </si>
+  <si>
+    <t>J'ai implementé la feature Login et Signin en fictif car nous n'avons pas de vrai backend. J'ai fais toutes les routes et l'IA m'a aidé pour le CSS.</t>
+  </si>
+  <si>
+    <t>J'ai régler un problèmes qu'il y avait avec la page des derniers ouvrages et la page details</t>
+  </si>
+  <si>
+    <t>J'ai commencé a faire la pages details mais depuis le catalogue pour avoir le details des livres depuis la page catalogue.</t>
+  </si>
+  <si>
+    <t>J'ai finaliser la pages details depuis catalogue, j'ai du implementer un nouveau props qui change le router link</t>
+  </si>
+  <si>
+    <t>J'ai fix le CSS de certaines pages car il y avait des bugs d'affichages</t>
+  </si>
+  <si>
+    <t>Le prof nous a expliqué comment fonctionnait les routes etc avec services.json</t>
+  </si>
+  <si>
+    <t>J'ai remplis mon JDT car je ne l'avais pas fais et j'ai effecué mes commits</t>
+  </si>
+  <si>
+    <t>Nous avons ensemble analyser notre code et nous avons trouver le problème qui bloquait déjà hier. Et nous avons réussi a reafficher les livres dynamiquement.</t>
+  </si>
+  <si>
+    <t>J'ai ajouté le html + le CSS pour les ajout de commentaires</t>
+  </si>
+  <si>
+    <t>J'ai commencé a faire la route pour l'ajout des commentaires et j'ai changé le .json pour que ça marche</t>
   </si>
 </sst>
 </file>
@@ -1166,19 +1214,19 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>25</c:v>
+                  <c:v>140</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>150</c:v>
+                  <c:v>780</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>50</c:v>
+                  <c:v>70</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>225</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2021,16 +2069,16 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.1111111111111111</c:v>
+                  <c:v>0.11522633744855967</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.66666666666666663</c:v>
+                  <c:v>0.64197530864197527</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.22222222222222221</c:v>
+                  <c:v>5.7613168724279837E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4265,7 +4313,7 @@
       <c r="B3" s="87"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>3 heures 45 minutes</v>
+        <v>20 heures 15 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4280,15 +4328,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>105</v>
+        <v>615</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>225</v>
+        <v>1215</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4426,15 +4474,23 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="63" t="str">
+      <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v/>
-      </c>
-      <c r="B11" s="34"/>
-      <c r="C11" s="35"/>
+        <v>7</v>
+      </c>
+      <c r="B11" s="34">
+        <v>46064</v>
+      </c>
+      <c r="C11" s="35">
+        <v>1</v>
+      </c>
       <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="23"/>
+      <c r="E11" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>36</v>
+      </c>
       <c r="G11" s="40"/>
       <c r="M11" t="s">
         <v>14</v>
@@ -4453,9 +4509,15 @@
       </c>
       <c r="B12" s="30"/>
       <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
+      <c r="D12" s="32">
+        <v>20</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>37</v>
+      </c>
       <c r="G12" s="39"/>
       <c r="M12" t="s">
         <v>18</v>
@@ -4473,10 +4535,18 @@
         <v/>
       </c>
       <c r="B13" s="34"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="C13" s="35">
+        <v>1</v>
+      </c>
+      <c r="D13" s="36">
+        <v>10</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4492,9 +4562,15 @@
       </c>
       <c r="B14" s="30"/>
       <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+      <c r="D14" s="32">
+        <v>30</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>39</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -4503,16 +4579,24 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="63" t="str">
+    <row r="15" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v/>
-      </c>
-      <c r="B15" s="34"/>
+        <v>9</v>
+      </c>
+      <c r="B15" s="34">
+        <v>46077</v>
+      </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>30</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>40</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -4521,31 +4605,45 @@
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A16" s="62" t="str">
         <f>IF(ISBLANK(B16),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B16))</f>
         <v/>
       </c>
       <c r="B16" s="30"/>
       <c r="C16" s="31"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="33"/>
-      <c r="F16" s="23"/>
+      <c r="D16" s="32">
+        <v>20</v>
+      </c>
+      <c r="E16" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G16" s="39"/>
       <c r="O16">
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A17" s="63" t="str">
         <f>IF(ISBLANK(B17),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B17))</f>
         <v/>
       </c>
       <c r="B17" s="34"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="36"/>
-      <c r="E17" s="37"/>
-      <c r="F17" s="23"/>
+      <c r="C17" s="35">
+        <v>1</v>
+      </c>
+      <c r="D17" s="36">
+        <v>45</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G17" s="40"/>
       <c r="O17">
         <v>45</v>
@@ -4558,39 +4656,59 @@
       </c>
       <c r="B18" s="30"/>
       <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="84"/>
+      <c r="D18" s="32">
+        <v>25</v>
+      </c>
+      <c r="E18" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F18" s="84" t="s">
+        <v>43</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="63" t="str">
         <f>IF(ISBLANK(B19),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B19))</f>
         <v/>
       </c>
       <c r="B19" s="34"/>
       <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="D19" s="36">
+        <v>45</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>44</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A20" s="62" t="str">
         <f>IF(ISBLANK(B20),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B20))</f>
         <v/>
       </c>
       <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="C20" s="31">
+        <v>1</v>
+      </c>
+      <c r="D20" s="32">
+        <v>45</v>
+      </c>
+      <c r="E20" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>45</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -4600,9 +4718,15 @@
       </c>
       <c r="B21" s="34"/>
       <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="D21" s="36">
+        <v>45</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>46</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -4612,9 +4736,15 @@
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
+      <c r="D22" s="32">
+        <v>20</v>
+      </c>
+      <c r="E22" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -4624,33 +4754,57 @@
       </c>
       <c r="B23" s="34"/>
       <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+      <c r="D23" s="36">
+        <v>10</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="62" t="str">
+      <c r="A24" s="62">
         <f>IF(ISBLANK(B24),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="30"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="33"/>
+        <v>10</v>
+      </c>
+      <c r="B24" s="30">
+        <v>46084</v>
+      </c>
+      <c r="C24" s="31">
+        <v>3</v>
+      </c>
+      <c r="D24" s="32">
+        <v>45</v>
+      </c>
+      <c r="E24" s="33" t="s">
+        <v>18</v>
+      </c>
       <c r="F24" s="23"/>
       <c r="G24" s="39"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="63" t="str">
+    <row r="25" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="63">
         <f>IF(ISBLANK(B25),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="34"/>
-      <c r="C25" s="35"/>
-      <c r="D25" s="36"/>
-      <c r="E25" s="37"/>
-      <c r="F25" s="23"/>
+        <v>10</v>
+      </c>
+      <c r="B25" s="34">
+        <v>46085</v>
+      </c>
+      <c r="C25" s="35">
+        <v>1</v>
+      </c>
+      <c r="D25" s="36">
+        <v>30</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="23" t="s">
+        <v>49</v>
+      </c>
       <c r="G25" s="40"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
@@ -4660,21 +4814,33 @@
       </c>
       <c r="B26" s="30"/>
       <c r="C26" s="31"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="33"/>
-      <c r="F26" s="23"/>
+      <c r="D26" s="32">
+        <v>45</v>
+      </c>
+      <c r="E26" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="23" t="s">
+        <v>50</v>
+      </c>
       <c r="G26" s="39"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A27" s="63" t="str">
         <f>IF(ISBLANK(B27),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B27))</f>
         <v/>
       </c>
       <c r="B27" s="34"/>
       <c r="C27" s="35"/>
-      <c r="D27" s="36"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="23"/>
+      <c r="D27" s="36">
+        <v>45</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F27" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G27" s="40"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
@@ -10875,11 +11041,11 @@
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>25</v>
+        <v>140</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10887,11 +11053,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 25 min</v>
+        <v>2 h 20 min</v>
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.1111111111111111</v>
+        <v>0.11522633744855967</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10908,15 +11074,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>120</v>
+        <v>420</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>30</v>
+        <v>360</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>150</v>
+        <v>780</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10924,11 +11090,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>2 h 30 min</v>
+        <v>13 h 00 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.66666666666666663</v>
+        <v>0.64197530864197527</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10986,11 +11152,11 @@
       </c>
       <c r="B9">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E9,'Journal de travail'!$D$7:$D$532)</f>
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="C9">
         <f t="shared" si="0"/>
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="E9" s="77" t="str">
         <f>'Journal de travail'!M11</f>
@@ -10998,11 +11164,11 @@
       </c>
       <c r="F9" s="74" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 50 min</v>
+        <v>1 h 10 min</v>
       </c>
       <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>0.22222222222222221</v>
+        <v>5.7613168724279837E-2</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11019,26 +11185,26 @@
     <row r="10" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E10,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="B10">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E10,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="C10">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E10" s="78" t="s">
         <v>18</v>
       </c>
       <c r="F10" s="79" t="str">
         <f t="shared" ref="F10" si="4">QUOTIENT(SUM(A10:B10),60)&amp;" h "&amp;TEXT(MOD(SUM(A10:B10),60), "00")&amp;" min"</f>
-        <v>0 h 00 min</v>
+        <v>3 h 45 min</v>
       </c>
       <c r="G10" s="80">
         <f>SUM(A10:B10)/$C$11</f>
-        <v>0</v>
+        <v>0.18518518518518517</v>
       </c>
       <c r="L10" s="69" t="s">
         <v>18</v>
@@ -11054,26 +11220,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>120</v>
+        <v>600</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>105</v>
+        <v>615</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>225</v>
+        <v>1215</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>3 h 45 min</v>
+        <v>20 h 15 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>4.1666666666666664E-2</v>
+        <v>0.22500000000000001</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>

</xml_diff>